<commit_message>
Add 24/25 5-man lineup data + team CSVs
</commit_message>
<xml_diff>
--- a/teamscore2425.csv.xlsx
+++ b/teamscore2425.csv.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/28b260e40b8dae5f/Desktop/All new stats data and references/oursafetynet/PBPselfscraped/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1E0EC615-E8A4-4E44-85C3-C882B3570875}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{727B1EE9-5DF8-47C1-A79A-896E9FC03029}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="20928" windowHeight="12432" xr2:uid="{47078471-CEDA-4F85-B4D2-8BE021C1124D}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="20928" windowHeight="12432" xr2:uid="{3AE021B5-4C67-4A79-A9AD-61EA38D9E391}"/>
   </bookViews>
   <sheets>
-    <sheet name="pbpstats_export (12)" sheetId="1" r:id="rId1"/>
+    <sheet name="pbpstats_export (11)" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -22,6 +22,9 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
+    <t>Name</t>
+  </si>
+  <si>
     <t>GamesPlayed</t>
   </si>
   <si>
@@ -191,9 +194,6 @@
   </si>
   <si>
     <t>SAS</t>
-  </si>
-  <si>
-    <t>te</t>
   </si>
 </sst>
 </file>
@@ -1053,99 +1053,99 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEE4970A-E291-4626-B87B-2981FEE618C6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BD5E114-E645-4743-BAFA-FDFE7674B1F4}">
   <dimension ref="A1:AB31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <sheetData>
     <row r="1" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
-        <v>57</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="O1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="R1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="S1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="T1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="U1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="V1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="W1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="X1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="Y1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Z1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AA1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AB1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B2">
         <v>82</v>
@@ -1154,22 +1154,22 @@
         <v>8083</v>
       </c>
       <c r="D2">
-        <v>113.70731707317</v>
+        <v>9324</v>
       </c>
       <c r="E2">
-        <v>25.304878048780399</v>
+        <v>2075</v>
       </c>
       <c r="F2">
-        <v>47.963414634146297</v>
+        <v>3933</v>
       </c>
       <c r="G2">
         <v>0.52758708365115603</v>
       </c>
       <c r="H2">
-        <v>15.414634146341401</v>
+        <v>1264</v>
       </c>
       <c r="I2">
-        <v>42.378048780487802</v>
+        <v>3475</v>
       </c>
       <c r="J2">
         <v>0.36374100719424401</v>
@@ -1178,19 +1178,19 @@
         <v>0.36566299942096098</v>
       </c>
       <c r="L2">
-        <v>16.8536585365853</v>
+        <v>1382</v>
       </c>
       <c r="M2">
-        <v>31.2439024390243</v>
+        <v>2562</v>
       </c>
       <c r="N2">
-        <v>19.365853658536501</v>
+        <v>1588</v>
       </c>
       <c r="O2">
-        <v>40.4268292682926</v>
+        <v>3315</v>
       </c>
       <c r="P2">
-        <v>5.8170731707316996</v>
+        <v>477</v>
       </c>
       <c r="Q2">
         <v>0.617349397590361</v>
@@ -1214,16 +1214,16 @@
         <v>0.56745208155292304</v>
       </c>
       <c r="X2">
-        <v>4.4634146341463401</v>
+        <v>366</v>
       </c>
       <c r="Y2">
-        <v>4.8048780487804796</v>
+        <v>394</v>
       </c>
       <c r="Z2">
         <v>0.100177981184846</v>
       </c>
       <c r="AA2">
-        <v>0.57317073170731703</v>
+        <v>47</v>
       </c>
       <c r="AB2">
         <v>1.3525179856115101E-2</v>
@@ -1231,7 +1231,7 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B3">
         <v>82</v>
@@ -1240,22 +1240,22 @@
         <v>7978</v>
       </c>
       <c r="D3">
-        <v>110.597560975609</v>
+        <v>9069</v>
       </c>
       <c r="E3">
-        <v>26.756097560975601</v>
+        <v>2194</v>
       </c>
       <c r="F3">
-        <v>49.707317073170699</v>
+        <v>4076</v>
       </c>
       <c r="G3">
         <v>0.53827281648675096</v>
       </c>
       <c r="H3">
-        <v>13.707317073170699</v>
+        <v>1124</v>
       </c>
       <c r="I3">
-        <v>37.317073170731703</v>
+        <v>3060</v>
       </c>
       <c r="J3">
         <v>0.36732026143790802</v>
@@ -1264,19 +1264,19 @@
         <v>0.36949375410913798</v>
       </c>
       <c r="L3">
-        <v>15.9634146341463</v>
+        <v>1309</v>
       </c>
       <c r="M3">
-        <v>28.9268292682926</v>
+        <v>2372</v>
       </c>
       <c r="N3">
-        <v>24.585365853658502</v>
+        <v>2016</v>
       </c>
       <c r="O3">
-        <v>35.8536585365853</v>
+        <v>2940</v>
       </c>
       <c r="P3">
-        <v>5.2682926829268197</v>
+        <v>432</v>
       </c>
       <c r="Q3">
         <v>0.54056517775752</v>
@@ -1300,16 +1300,16 @@
         <v>0.57598570881714894</v>
       </c>
       <c r="X3">
-        <v>4.1219512195121899</v>
+        <v>338</v>
       </c>
       <c r="Y3">
-        <v>4.1951219512195097</v>
+        <v>344</v>
       </c>
       <c r="Z3">
         <v>8.4396467124631905E-2</v>
       </c>
       <c r="AA3">
-        <v>0.46341463414634099</v>
+        <v>38</v>
       </c>
       <c r="AB3">
         <v>1.2418300653594699E-2</v>
@@ -1317,7 +1317,7 @@
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B4">
         <v>82</v>
@@ -1326,22 +1326,22 @@
         <v>8428</v>
       </c>
       <c r="D4">
-        <v>118.10975609755999</v>
+        <v>9685</v>
       </c>
       <c r="E4">
-        <v>29.829268292682901</v>
+        <v>2446</v>
       </c>
       <c r="F4">
-        <v>54.097560975609703</v>
+        <v>4436</v>
       </c>
       <c r="G4">
         <v>0.55139765554553599</v>
       </c>
       <c r="H4">
-        <v>13.5</v>
+        <v>1107</v>
       </c>
       <c r="I4">
-        <v>37.670731707317003</v>
+        <v>3089</v>
       </c>
       <c r="J4">
         <v>0.35836840401424402</v>
@@ -1350,19 +1350,19 @@
         <v>0.36084828711256101</v>
       </c>
       <c r="L4">
-        <v>17.951219512195099</v>
+        <v>1472</v>
       </c>
       <c r="M4">
-        <v>37.170731707317003</v>
+        <v>3048</v>
       </c>
       <c r="N4">
-        <v>22.487804878048699</v>
+        <v>1844</v>
       </c>
       <c r="O4">
-        <v>33</v>
+        <v>2706</v>
       </c>
       <c r="P4">
-        <v>7.5</v>
+        <v>615</v>
       </c>
       <c r="Q4">
         <v>0.62305805396565805</v>
@@ -1386,16 +1386,16 @@
         <v>0.57862879060289996</v>
       </c>
       <c r="X4">
-        <v>5.1707317073170698</v>
+        <v>424</v>
       </c>
       <c r="Y4">
-        <v>4.6341463414634099</v>
+        <v>380</v>
       </c>
       <c r="Z4">
         <v>8.5662759242560796E-2</v>
       </c>
       <c r="AA4">
-        <v>0.292682926829268</v>
+        <v>24</v>
       </c>
       <c r="AB4">
         <v>7.76950469407575E-3</v>
@@ -1403,7 +1403,7 @@
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B5">
         <v>82</v>
@@ -1412,22 +1412,22 @@
         <v>8241</v>
       </c>
       <c r="D5">
-        <v>117.365853658536</v>
+        <v>9624</v>
       </c>
       <c r="E5">
-        <v>30.402439024390201</v>
+        <v>2493</v>
       </c>
       <c r="F5">
-        <v>53.560975609756099</v>
+        <v>4392</v>
       </c>
       <c r="G5">
         <v>0.56762295081967196</v>
       </c>
       <c r="H5">
-        <v>13.182926829268199</v>
+        <v>1081</v>
       </c>
       <c r="I5">
-        <v>35.780487804878</v>
+        <v>2934</v>
       </c>
       <c r="J5">
         <v>0.36843899113837703</v>
@@ -1436,19 +1436,19 @@
         <v>0.37122252747252699</v>
       </c>
       <c r="L5">
-        <v>17.012195121951201</v>
+        <v>1395</v>
       </c>
       <c r="M5">
-        <v>36.292682926829201</v>
+        <v>2976</v>
       </c>
       <c r="N5">
-        <v>24.512195121951201</v>
+        <v>2010</v>
       </c>
       <c r="O5">
-        <v>33.292682926829201</v>
+        <v>2730</v>
       </c>
       <c r="P5">
-        <v>6.2560975609755998</v>
+        <v>513</v>
       </c>
       <c r="Q5">
         <v>0.59687123947051701</v>
@@ -1472,16 +1472,16 @@
         <v>0.59261089830717895</v>
       </c>
       <c r="X5">
-        <v>4.1951219512195097</v>
+        <v>344</v>
       </c>
       <c r="Y5">
-        <v>4.1341463414634099</v>
+        <v>339</v>
       </c>
       <c r="Z5">
         <v>7.7185792349726695E-2</v>
       </c>
       <c r="AA5">
-        <v>0.32926829268292601</v>
+        <v>27</v>
       </c>
       <c r="AB5">
         <v>9.2024539877300603E-3</v>
@@ -1489,7 +1489,7 @@
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B6">
         <v>82</v>
@@ -1498,22 +1498,22 @@
         <v>8421</v>
       </c>
       <c r="D6">
-        <v>121.63414634146299</v>
+        <v>9974</v>
       </c>
       <c r="E6">
-        <v>30.804878048780399</v>
+        <v>2526</v>
       </c>
       <c r="F6">
-        <v>55.402439024390198</v>
+        <v>4543</v>
       </c>
       <c r="G6">
         <v>0.556020250935505</v>
       </c>
       <c r="H6">
-        <v>13.914634146341401</v>
+        <v>1141</v>
       </c>
       <c r="I6">
-        <v>37.890243902439003</v>
+        <v>3107</v>
       </c>
       <c r="J6">
         <v>0.36723527518506599</v>
@@ -1522,19 +1522,19 @@
         <v>0.37025008119519298</v>
       </c>
       <c r="L6">
-        <v>18.280487804878</v>
+        <v>1499</v>
       </c>
       <c r="M6">
-        <v>32.487804878048699</v>
+        <v>2664</v>
       </c>
       <c r="N6">
-        <v>29.121951219512098</v>
+        <v>2388</v>
       </c>
       <c r="O6">
-        <v>36.475609756097498</v>
+        <v>2991</v>
       </c>
       <c r="P6">
-        <v>5.2682926829268197</v>
+        <v>432</v>
       </c>
       <c r="Q6">
         <v>0.52731591448931103</v>
@@ -1558,16 +1558,16 @@
         <v>0.58772759517616402</v>
       </c>
       <c r="X6">
-        <v>5.7073170731707297</v>
+        <v>468</v>
       </c>
       <c r="Y6">
-        <v>5.2317073170731696</v>
+        <v>429</v>
       </c>
       <c r="Z6">
         <v>9.4430992736077399E-2</v>
       </c>
       <c r="AA6">
-        <v>0.26829268292682901</v>
+        <v>22</v>
       </c>
       <c r="AB6">
         <v>7.08078532346314E-3</v>
@@ -1575,7 +1575,7 @@
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B7">
         <v>82</v>
@@ -1584,22 +1584,22 @@
         <v>8003</v>
       </c>
       <c r="D7">
-        <v>105.097560975609</v>
+        <v>8618</v>
       </c>
       <c r="E7">
-        <v>25.329268292682901</v>
+        <v>2077</v>
       </c>
       <c r="F7">
-        <v>50.768292682926798</v>
+        <v>4163</v>
       </c>
       <c r="G7">
         <v>0.49891904876291099</v>
       </c>
       <c r="H7">
-        <v>12.987804878048699</v>
+        <v>1065</v>
       </c>
       <c r="I7">
-        <v>38.329268292682897</v>
+        <v>3143</v>
       </c>
       <c r="J7">
         <v>0.33884823417117399</v>
@@ -1608,19 +1608,19 @@
         <v>0.341565105837075</v>
       </c>
       <c r="L7">
-        <v>15.4756097560975</v>
+        <v>1269</v>
       </c>
       <c r="M7">
-        <v>27.365853658536501</v>
+        <v>2244</v>
       </c>
       <c r="N7">
-        <v>23.292682926829201</v>
+        <v>1910</v>
       </c>
       <c r="O7">
-        <v>31.902439024390201</v>
+        <v>2616</v>
       </c>
       <c r="P7">
-        <v>7.0609756097560901</v>
+        <v>579</v>
       </c>
       <c r="Q7">
         <v>0.54020221473278696</v>
@@ -1644,16 +1644,16 @@
         <v>0.53645898364340106</v>
       </c>
       <c r="X7">
-        <v>4.8292682926829196</v>
+        <v>396</v>
       </c>
       <c r="Y7">
-        <v>4.8292682926829196</v>
+        <v>396</v>
       </c>
       <c r="Z7">
         <v>9.5123708863800102E-2</v>
       </c>
       <c r="AA7">
-        <v>0.47560975609756001</v>
+        <v>39</v>
       </c>
       <c r="AB7">
         <v>1.24085268851415E-2</v>
@@ -1661,7 +1661,7 @@
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B8">
         <v>82</v>
@@ -1670,22 +1670,22 @@
         <v>8181</v>
       </c>
       <c r="D8">
-        <v>115.451219512195</v>
+        <v>9467</v>
       </c>
       <c r="E8">
-        <v>29.878048780487799</v>
+        <v>2450</v>
       </c>
       <c r="F8">
-        <v>54.390243902439003</v>
+        <v>4460</v>
       </c>
       <c r="G8">
         <v>0.54932735426008905</v>
       </c>
       <c r="H8">
-        <v>12.8170731707317</v>
+        <v>1051</v>
       </c>
       <c r="I8">
-        <v>35.378048780487802</v>
+        <v>2901</v>
       </c>
       <c r="J8">
         <v>0.362288865908307</v>
@@ -1694,19 +1694,19 @@
         <v>0.365057311566516</v>
       </c>
       <c r="L8">
-        <v>17.2439024390243</v>
+        <v>1414</v>
       </c>
       <c r="M8">
-        <v>30.902439024390201</v>
+        <v>2534</v>
       </c>
       <c r="N8">
-        <v>28.8536585365853</v>
+        <v>2366</v>
       </c>
       <c r="O8">
-        <v>32.817073170731703</v>
+        <v>2691</v>
       </c>
       <c r="P8">
-        <v>5.6341463414634099</v>
+        <v>462</v>
       </c>
       <c r="Q8">
         <v>0.51714285714285702</v>
@@ -1730,16 +1730,16 @@
         <v>0.57934849416103196</v>
       </c>
       <c r="X8">
-        <v>5.9024390243902403</v>
+        <v>484</v>
       </c>
       <c r="Y8">
-        <v>4.7439024390243896</v>
+        <v>389</v>
       </c>
       <c r="Z8">
         <v>8.7219730941704002E-2</v>
       </c>
       <c r="AA8">
-        <v>0.28048780487804797</v>
+        <v>23</v>
       </c>
       <c r="AB8">
         <v>7.9283005860048203E-3</v>
@@ -1747,7 +1747,7 @@
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B9">
         <v>82</v>
@@ -1756,22 +1756,22 @@
         <v>8149</v>
       </c>
       <c r="D9">
-        <v>115.512195121951</v>
+        <v>9472</v>
       </c>
       <c r="E9">
-        <v>27.8536585365853</v>
+        <v>2284</v>
       </c>
       <c r="F9">
-        <v>49.743902439024303</v>
+        <v>4079</v>
       </c>
       <c r="G9">
         <v>0.55994116204952105</v>
       </c>
       <c r="H9">
-        <v>14.1585365853658</v>
+        <v>1161</v>
       </c>
       <c r="I9">
-        <v>36.621951219512198</v>
+        <v>3003</v>
       </c>
       <c r="J9">
         <v>0.38661338661338601</v>
@@ -1780,19 +1780,19 @@
         <v>0.38775510204081598</v>
       </c>
       <c r="L9">
-        <v>17.329268292682901</v>
+        <v>1421</v>
       </c>
       <c r="M9">
-        <v>26.707317073170699</v>
+        <v>2190</v>
       </c>
       <c r="N9">
-        <v>29</v>
+        <v>2378</v>
       </c>
       <c r="O9">
-        <v>36.402439024390198</v>
+        <v>2985</v>
       </c>
       <c r="P9">
-        <v>6.07317073170731</v>
+        <v>498</v>
       </c>
       <c r="Q9">
         <v>0.47942206654991198</v>
@@ -1816,16 +1816,16 @@
         <v>0.599454522389953</v>
       </c>
       <c r="X9">
-        <v>3.9024390243902398</v>
+        <v>320</v>
       </c>
       <c r="Y9">
-        <v>3.5365853658536501</v>
+        <v>290</v>
       </c>
       <c r="Z9">
         <v>7.1095856827653806E-2</v>
       </c>
       <c r="AA9">
-        <v>0.30487804878048702</v>
+        <v>25</v>
       </c>
       <c r="AB9">
         <v>8.3250083250083207E-3</v>
@@ -1833,7 +1833,7 @@
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B10">
         <v>82</v>
@@ -1842,22 +1842,22 @@
         <v>8012</v>
       </c>
       <c r="D10">
-        <v>109.60975609755999</v>
+        <v>8988</v>
       </c>
       <c r="E10">
-        <v>26.987804878048699</v>
+        <v>2213</v>
       </c>
       <c r="F10">
-        <v>50.219512195121901</v>
+        <v>4118</v>
       </c>
       <c r="G10">
         <v>0.53739679456046596</v>
       </c>
       <c r="H10">
-        <v>12.6951219512195</v>
+        <v>1041</v>
       </c>
       <c r="I10">
-        <v>37.195121951219498</v>
+        <v>3050</v>
       </c>
       <c r="J10">
         <v>0.34131147540983597</v>
@@ -1866,19 +1866,19 @@
         <v>0.34458788480635499</v>
       </c>
       <c r="L10">
-        <v>17.548780487804802</v>
+        <v>1439</v>
       </c>
       <c r="M10">
-        <v>26.170731707317</v>
+        <v>2146</v>
       </c>
       <c r="N10">
-        <v>27.804878048780399</v>
+        <v>2280</v>
       </c>
       <c r="O10">
-        <v>30.292682926829201</v>
+        <v>2484</v>
       </c>
       <c r="P10">
-        <v>7.7926829268292597</v>
+        <v>639</v>
       </c>
       <c r="Q10">
         <v>0.484862178038861</v>
@@ -1902,16 +1902,16 @@
         <v>0.56250784486004701</v>
       </c>
       <c r="X10">
-        <v>4.6097560975609699</v>
+        <v>378</v>
       </c>
       <c r="Y10">
-        <v>4.8048780487804796</v>
+        <v>394</v>
       </c>
       <c r="Z10">
         <v>9.5677513355998001E-2</v>
       </c>
       <c r="AA10">
-        <v>0.31707317073170699</v>
+        <v>26</v>
       </c>
       <c r="AB10">
         <v>8.5245901639344202E-3</v>
@@ -1919,7 +1919,7 @@
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B11">
         <v>82</v>
@@ -1928,22 +1928,22 @@
         <v>8141</v>
       </c>
       <c r="D11">
-        <v>109.829268292682</v>
+        <v>9006</v>
       </c>
       <c r="E11">
-        <v>28.609756097560901</v>
+        <v>2346</v>
       </c>
       <c r="F11">
-        <v>55.231707317073102</v>
+        <v>4529</v>
       </c>
       <c r="G11">
         <v>0.51799514241554401</v>
       </c>
       <c r="H11">
-        <v>12.024390243902401</v>
+        <v>986</v>
       </c>
       <c r="I11">
-        <v>34.621951219512198</v>
+        <v>2839</v>
       </c>
       <c r="J11">
         <v>0.34730538922155602</v>
@@ -1952,19 +1952,19 @@
         <v>0.34828682444365899</v>
       </c>
       <c r="L11">
-        <v>16.5365853658536</v>
+        <v>1356</v>
       </c>
       <c r="M11">
-        <v>31.609756097560901</v>
+        <v>2592</v>
       </c>
       <c r="N11">
-        <v>25.609756097560901</v>
+        <v>2100</v>
       </c>
       <c r="O11">
-        <v>30.109756097560901</v>
+        <v>2469</v>
       </c>
       <c r="P11">
-        <v>5.9634146341463401</v>
+        <v>489</v>
       </c>
       <c r="Q11">
         <v>0.55242966751918099</v>
@@ -1988,16 +1988,16 @@
         <v>0.55068106516136905</v>
       </c>
       <c r="X11">
-        <v>5.3658536585365804</v>
+        <v>440</v>
       </c>
       <c r="Y11">
-        <v>4.8902439024390203</v>
+        <v>401</v>
       </c>
       <c r="Z11">
         <v>8.8540516670346597E-2</v>
       </c>
       <c r="AA11">
-        <v>0.32926829268292601</v>
+        <v>27</v>
       </c>
       <c r="AB11">
         <v>9.5103909827404E-3</v>
@@ -2005,7 +2005,7 @@
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B12">
         <v>82</v>
@@ -2014,22 +2014,22 @@
         <v>7914</v>
       </c>
       <c r="D12">
-        <v>116.268292682926</v>
+        <v>9534</v>
       </c>
       <c r="E12">
-        <v>23.8536585365853</v>
+        <v>1956</v>
       </c>
       <c r="F12">
-        <v>41.792682926829201</v>
+        <v>3427</v>
       </c>
       <c r="G12">
         <v>0.57076159906623802</v>
       </c>
       <c r="H12">
-        <v>17.768292682926798</v>
+        <v>1457</v>
       </c>
       <c r="I12">
-        <v>48.231707317073102</v>
+        <v>3955</v>
       </c>
       <c r="J12">
         <v>0.36839443742098599</v>
@@ -2038,19 +2038,19 @@
         <v>0.36979695431471998</v>
       </c>
       <c r="L12">
-        <v>15.256097560975601</v>
+        <v>1251</v>
       </c>
       <c r="M12">
-        <v>24.0731707317073</v>
+        <v>1974</v>
       </c>
       <c r="N12">
-        <v>23.634146341463399</v>
+        <v>1938</v>
       </c>
       <c r="O12">
-        <v>42.329268292682897</v>
+        <v>3471</v>
       </c>
       <c r="P12">
-        <v>10.9756097560975</v>
+        <v>900</v>
       </c>
       <c r="Q12">
         <v>0.504601226993865</v>
@@ -2074,16 +2074,16 @@
         <v>0.58978654753040405</v>
       </c>
       <c r="X12">
-        <v>3.9268292682926802</v>
+        <v>322</v>
       </c>
       <c r="Y12">
-        <v>3.1463414634146298</v>
+        <v>258</v>
       </c>
       <c r="Z12">
         <v>7.52845053983075E-2</v>
       </c>
       <c r="AA12">
-        <v>0.45121951219512102</v>
+        <v>37</v>
       </c>
       <c r="AB12">
         <v>9.35524652338811E-3</v>
@@ -2091,7 +2091,7 @@
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B13">
         <v>82</v>
@@ -2100,22 +2100,22 @@
         <v>8145</v>
       </c>
       <c r="D13">
-        <v>114.170731707317</v>
+        <v>9362</v>
       </c>
       <c r="E13">
-        <v>29.5365853658536</v>
+        <v>2422</v>
       </c>
       <c r="F13">
-        <v>53.560975609756099</v>
+        <v>4392</v>
       </c>
       <c r="G13">
         <v>0.55145719489981704</v>
       </c>
       <c r="H13">
-        <v>12.439024390243899</v>
+        <v>1020</v>
       </c>
       <c r="I13">
-        <v>34.158536585365802</v>
+        <v>2801</v>
       </c>
       <c r="J13">
         <v>0.364155658693323</v>
@@ -2124,19 +2124,19 @@
         <v>0.36664270309130098</v>
       </c>
       <c r="L13">
-        <v>17.780487804878</v>
+        <v>1458</v>
       </c>
       <c r="M13">
-        <v>30.439024390243901</v>
+        <v>2496</v>
       </c>
       <c r="N13">
-        <v>28.634146341463399</v>
+        <v>2348</v>
       </c>
       <c r="O13">
-        <v>30.0731707317073</v>
+        <v>2466</v>
       </c>
       <c r="P13">
-        <v>7.2439024390243896</v>
+        <v>594</v>
       </c>
       <c r="Q13">
         <v>0.51527663088356701</v>
@@ -2160,16 +2160,16 @@
         <v>0.58310422394401396</v>
       </c>
       <c r="X13">
-        <v>4.48780487804878</v>
+        <v>368</v>
       </c>
       <c r="Y13">
-        <v>4.2804878048780397</v>
+        <v>351</v>
       </c>
       <c r="Z13">
         <v>7.9918032786885196E-2</v>
       </c>
       <c r="AA13">
-        <v>0.292682926829268</v>
+        <v>24</v>
       </c>
       <c r="AB13">
         <v>8.5683684398429102E-3</v>
@@ -2177,7 +2177,7 @@
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B14">
         <v>82</v>
@@ -2186,22 +2186,22 @@
         <v>7993</v>
       </c>
       <c r="D14">
-        <v>115.63414634146299</v>
+        <v>9482</v>
       </c>
       <c r="E14">
-        <v>30.682926829268201</v>
+        <v>2516</v>
       </c>
       <c r="F14">
-        <v>55.060975609756099</v>
+        <v>4515</v>
       </c>
       <c r="G14">
         <v>0.55725359911406402</v>
       </c>
       <c r="H14">
-        <v>12.5731707317073</v>
+        <v>1031</v>
       </c>
       <c r="I14">
-        <v>34.0731707317073</v>
+        <v>2794</v>
       </c>
       <c r="J14">
         <v>0.36900501073729403</v>
@@ -2210,19 +2210,19 @@
         <v>0.37166546503244402</v>
       </c>
       <c r="L14">
-        <v>16.548780487804802</v>
+        <v>1357</v>
       </c>
       <c r="M14">
-        <v>34.048780487804798</v>
+        <v>2792</v>
       </c>
       <c r="N14">
-        <v>27.3170731707317</v>
+        <v>2240</v>
       </c>
       <c r="O14">
-        <v>31.2439024390243</v>
+        <v>2562</v>
       </c>
       <c r="P14">
-        <v>6.4756097560975601</v>
+        <v>531</v>
       </c>
       <c r="Q14">
         <v>0.554848966613672</v>
@@ -2246,16 +2246,16 @@
         <v>0.58898305084745695</v>
       </c>
       <c r="X14">
-        <v>5.3414634146341404</v>
+        <v>438</v>
       </c>
       <c r="Y14">
-        <v>4.6585365853658498</v>
+        <v>382</v>
       </c>
       <c r="Z14">
         <v>8.4606866002214801E-2</v>
       </c>
       <c r="AA14">
-        <v>0.292682926829268</v>
+        <v>24</v>
       </c>
       <c r="AB14">
         <v>8.5898353614889001E-3</v>
@@ -2263,7 +2263,7 @@
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B15">
         <v>82</v>
@@ -2272,22 +2272,22 @@
         <v>8105</v>
       </c>
       <c r="D15">
-        <v>115.731707317073</v>
+        <v>9490</v>
       </c>
       <c r="E15">
-        <v>30.451219512195099</v>
+        <v>2497</v>
       </c>
       <c r="F15">
-        <v>54.8536585365853</v>
+        <v>4498</v>
       </c>
       <c r="G15">
         <v>0.55513561582925697</v>
       </c>
       <c r="H15">
-        <v>12.5853658536585</v>
+        <v>1032</v>
       </c>
       <c r="I15">
-        <v>35.207317073170699</v>
+        <v>2887</v>
       </c>
       <c r="J15">
         <v>0.357464496016626</v>
@@ -2296,19 +2296,19 @@
         <v>0.35935866155454799</v>
       </c>
       <c r="L15">
-        <v>17.0731707317073</v>
+        <v>1400</v>
       </c>
       <c r="M15">
-        <v>31.121951219512098</v>
+        <v>2552</v>
       </c>
       <c r="N15">
-        <v>29.780487804878</v>
+        <v>2442</v>
       </c>
       <c r="O15">
-        <v>32.670731707317003</v>
+        <v>2679</v>
       </c>
       <c r="P15">
-        <v>5.08536585365853</v>
+        <v>417</v>
       </c>
       <c r="Q15">
         <v>0.51101321585903003</v>
@@ -2332,16 +2332,16 @@
         <v>0.581754429133858</v>
       </c>
       <c r="X15">
-        <v>5.09756097560975</v>
+        <v>418</v>
       </c>
       <c r="Y15">
-        <v>4.0121951219512102</v>
+        <v>329</v>
       </c>
       <c r="Z15">
         <v>7.3143619386393896E-2</v>
       </c>
       <c r="AA15">
-        <v>0.25609756097560898</v>
+        <v>21</v>
       </c>
       <c r="AB15">
         <v>7.2739868375476203E-3</v>
@@ -2349,7 +2349,7 @@
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B16">
         <v>82</v>
@@ -2358,22 +2358,22 @@
         <v>8435</v>
       </c>
       <c r="D16">
-        <v>117.80487804878</v>
+        <v>9660</v>
       </c>
       <c r="E16">
-        <v>27.768292682926798</v>
+        <v>2277</v>
       </c>
       <c r="F16">
-        <v>49.975609756097498</v>
+        <v>4098</v>
       </c>
       <c r="G16">
         <v>0.55563689604685196</v>
       </c>
       <c r="H16">
-        <v>15.439024390243899</v>
+        <v>1266</v>
       </c>
       <c r="I16">
-        <v>42.036585365853597</v>
+        <v>3447</v>
       </c>
       <c r="J16">
         <v>0.367275892080069</v>
@@ -2382,19 +2382,19 @@
         <v>0.368513119533527</v>
       </c>
       <c r="L16">
-        <v>15.951219512195101</v>
+        <v>1308</v>
       </c>
       <c r="M16">
-        <v>31.512195121951201</v>
+        <v>2584</v>
       </c>
       <c r="N16">
-        <v>24.024390243902399</v>
+        <v>1970</v>
       </c>
       <c r="O16">
-        <v>39.914634146341399</v>
+        <v>3273</v>
       </c>
       <c r="P16">
-        <v>6.4024390243902403</v>
+        <v>525</v>
       </c>
       <c r="Q16">
         <v>0.56741326306543605</v>
@@ -2418,16 +2418,16 @@
         <v>0.58436438622028097</v>
       </c>
       <c r="X16">
-        <v>4.2195121951219496</v>
+        <v>346</v>
       </c>
       <c r="Y16">
-        <v>4.7926829268292597</v>
+        <v>393</v>
       </c>
       <c r="Z16">
         <v>9.5900439238653004E-2</v>
       </c>
       <c r="AA16">
-        <v>0.292682926829268</v>
+        <v>24</v>
       </c>
       <c r="AB16">
         <v>6.96257615317667E-3</v>
@@ -2435,7 +2435,7 @@
     </row>
     <row r="17" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B17">
         <v>82</v>
@@ -2444,22 +2444,22 @@
         <v>8221</v>
       </c>
       <c r="D17">
-        <v>120.75609756097499</v>
+        <v>9902</v>
       </c>
       <c r="E17">
-        <v>33.414634146341399</v>
+        <v>2740</v>
       </c>
       <c r="F17">
-        <v>57.817073170731703</v>
+        <v>4741</v>
       </c>
       <c r="G17">
         <v>0.57793714406243402</v>
       </c>
       <c r="H17">
-        <v>12</v>
+        <v>984</v>
       </c>
       <c r="I17">
-        <v>31.9268292682926</v>
+        <v>2618</v>
       </c>
       <c r="J17">
         <v>0.37585943468296401</v>
@@ -2468,19 +2468,19 @@
         <v>0.38076773943388897</v>
       </c>
       <c r="L17">
-        <v>17.9268292682926</v>
+        <v>1470</v>
       </c>
       <c r="M17">
-        <v>41.707317073170699</v>
+        <v>3420</v>
       </c>
       <c r="N17">
-        <v>25.121951219512098</v>
+        <v>2060</v>
       </c>
       <c r="O17">
-        <v>30.439024390243901</v>
+        <v>2496</v>
       </c>
       <c r="P17">
-        <v>5.5609756097560901</v>
+        <v>456</v>
       </c>
       <c r="Q17">
         <v>0.62408759124087498</v>
@@ -2504,16 +2504,16 @@
         <v>0.60264860246551899</v>
       </c>
       <c r="X17">
-        <v>6.3658536585365804</v>
+        <v>522</v>
       </c>
       <c r="Y17">
-        <v>4.9634146341463401</v>
+        <v>407</v>
       </c>
       <c r="Z17">
         <v>8.5846867749419895E-2</v>
       </c>
       <c r="AA17">
-        <v>0.15853658536585299</v>
+        <v>13</v>
       </c>
       <c r="AB17">
         <v>4.9656226126814302E-3</v>
@@ -2521,7 +2521,7 @@
     </row>
     <row r="18" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B18">
         <v>82</v>
@@ -2530,22 +2530,22 @@
         <v>8211</v>
       </c>
       <c r="D18">
-        <v>120.475609756097</v>
+        <v>9879</v>
       </c>
       <c r="E18">
-        <v>30.085365853658502</v>
+        <v>2467</v>
       </c>
       <c r="F18">
-        <v>53.841463414634099</v>
+        <v>4415</v>
       </c>
       <c r="G18">
         <v>0.55877689694224197</v>
       </c>
       <c r="H18">
-        <v>14.5365853658536</v>
+        <v>1192</v>
       </c>
       <c r="I18">
-        <v>38.829268292682897</v>
+        <v>3184</v>
       </c>
       <c r="J18">
         <v>0.37437185929648198</v>
@@ -2554,19 +2554,19 @@
         <v>0.375</v>
       </c>
       <c r="L18">
-        <v>16.695121951219502</v>
+        <v>1369</v>
       </c>
       <c r="M18">
-        <v>29</v>
+        <v>2378</v>
       </c>
       <c r="N18">
-        <v>31.170731707317</v>
+        <v>2556</v>
       </c>
       <c r="O18">
-        <v>37.024390243902403</v>
+        <v>3036</v>
       </c>
       <c r="P18">
-        <v>6.58536585365853</v>
+        <v>540</v>
       </c>
       <c r="Q18">
         <v>0.48196189704094</v>
@@ -2590,16 +2590,16 @@
         <v>0.59170174383644003</v>
       </c>
       <c r="X18">
-        <v>3.58536585365853</v>
+        <v>294</v>
       </c>
       <c r="Y18">
-        <v>4.4512195121951201</v>
+        <v>365</v>
       </c>
       <c r="Z18">
         <v>8.2672706681766697E-2</v>
       </c>
       <c r="AA18">
-        <v>0.32926829268292601</v>
+        <v>27</v>
       </c>
       <c r="AB18">
         <v>8.4798994974874305E-3</v>
@@ -2607,7 +2607,7 @@
     </row>
     <row r="19" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B19">
         <v>82</v>
@@ -2616,22 +2616,22 @@
         <v>8277</v>
       </c>
       <c r="D19">
-        <v>108</v>
+        <v>8856</v>
       </c>
       <c r="E19">
-        <v>26.3170731707317</v>
+        <v>2158</v>
       </c>
       <c r="F19">
-        <v>50.731707317073102</v>
+        <v>4160</v>
       </c>
       <c r="G19">
         <v>0.51875000000000004</v>
       </c>
       <c r="H19">
-        <v>13.109756097560901</v>
+        <v>1075</v>
       </c>
       <c r="I19">
-        <v>39.146341463414601</v>
+        <v>3210</v>
       </c>
       <c r="J19">
         <v>0.33489096573208699</v>
@@ -2640,19 +2640,19 @@
         <v>0.33730781299027202</v>
       </c>
       <c r="L19">
-        <v>16.0365853658536</v>
+        <v>1315</v>
       </c>
       <c r="M19">
-        <v>28.878048780487799</v>
+        <v>2368</v>
       </c>
       <c r="N19">
-        <v>23.756097560975601</v>
+        <v>1948</v>
       </c>
       <c r="O19">
-        <v>31.975609756097501</v>
+        <v>2622</v>
       </c>
       <c r="P19">
-        <v>7.3536585365853604</v>
+        <v>603</v>
       </c>
       <c r="Q19">
         <v>0.54865616311399401</v>
@@ -2676,16 +2676,16 @@
         <v>0.54472547809993799</v>
       </c>
       <c r="X19">
-        <v>5.2195121951219496</v>
+        <v>428</v>
       </c>
       <c r="Y19">
-        <v>4.8292682926829196</v>
+        <v>396</v>
       </c>
       <c r="Z19">
         <v>9.5192307692307604E-2</v>
       </c>
       <c r="AA19">
-        <v>0.37804878048780399</v>
+        <v>31</v>
       </c>
       <c r="AB19">
         <v>9.6573208722741406E-3</v>
@@ -2693,7 +2693,7 @@
     </row>
     <row r="20" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B20">
         <v>82</v>
@@ -2702,22 +2702,22 @@
         <v>8199</v>
       </c>
       <c r="D20">
-        <v>121.93902439024301</v>
+        <v>9999</v>
       </c>
       <c r="E20">
-        <v>28.646341463414601</v>
+        <v>2349</v>
       </c>
       <c r="F20">
-        <v>49.304878048780402</v>
+        <v>4043</v>
       </c>
       <c r="G20">
         <v>0.58100420479841697</v>
       </c>
       <c r="H20">
-        <v>15.890243902439</v>
+        <v>1303</v>
       </c>
       <c r="I20">
-        <v>41.475609756097498</v>
+        <v>3401</v>
       </c>
       <c r="J20">
         <v>0.38312261099676498</v>
@@ -2726,19 +2726,19 @@
         <v>0.38452451269935001</v>
       </c>
       <c r="L20">
-        <v>16.975609756097501</v>
+        <v>1392</v>
       </c>
       <c r="M20">
-        <v>31.292682926829201</v>
+        <v>2566</v>
       </c>
       <c r="N20">
-        <v>26</v>
+        <v>2132</v>
       </c>
       <c r="O20">
-        <v>37.3536585365853</v>
+        <v>3063</v>
       </c>
       <c r="P20">
-        <v>10.3170731707317</v>
+        <v>846</v>
       </c>
       <c r="Q20">
         <v>0.54618986802894798</v>
@@ -2762,16 +2762,16 @@
         <v>0.60708201508882897</v>
       </c>
       <c r="X20">
-        <v>4.1463414634146298</v>
+        <v>340</v>
       </c>
       <c r="Y20">
-        <v>4.1097560975609699</v>
+        <v>337</v>
       </c>
       <c r="Z20">
         <v>8.3353945090279394E-2</v>
       </c>
       <c r="AA20">
-        <v>0.292682926829268</v>
+        <v>24</v>
       </c>
       <c r="AB20">
         <v>7.0567480152896201E-3</v>
@@ -2779,7 +2779,7 @@
     </row>
     <row r="21" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B21">
         <v>82</v>
@@ -2788,22 +2788,22 @@
         <v>8089</v>
       </c>
       <c r="D21">
-        <v>114.219512195121</v>
+        <v>9366</v>
       </c>
       <c r="E21">
-        <v>29.792682926829201</v>
+        <v>2443</v>
       </c>
       <c r="F21">
-        <v>57.524390243902403</v>
+        <v>4717</v>
       </c>
       <c r="G21">
         <v>0.51791392834428596</v>
       </c>
       <c r="H21">
-        <v>12.6585365853658</v>
+        <v>1038</v>
       </c>
       <c r="I21">
-        <v>35.829268292682897</v>
+        <v>2938</v>
       </c>
       <c r="J21">
         <v>0.35330156569094601</v>
@@ -2812,19 +2812,19 @@
         <v>0.35535775419376903</v>
       </c>
       <c r="L21">
-        <v>16.658536585365798</v>
+        <v>1366</v>
       </c>
       <c r="M21">
-        <v>26.682926829268201</v>
+        <v>2188</v>
       </c>
       <c r="N21">
-        <v>32.902439024390198</v>
+        <v>2698</v>
       </c>
       <c r="O21">
-        <v>30</v>
+        <v>2460</v>
       </c>
       <c r="P21">
-        <v>7.9756097560975601</v>
+        <v>654</v>
       </c>
       <c r="Q21">
         <v>0.44781006958657299</v>
@@ -2848,16 +2848,16 @@
         <v>0.55157559306030901</v>
       </c>
       <c r="X21">
-        <v>6.8048780487804796</v>
+        <v>558</v>
       </c>
       <c r="Y21">
-        <v>5.3414634146341404</v>
+        <v>438</v>
       </c>
       <c r="Z21">
         <v>9.2855628577485694E-2</v>
       </c>
       <c r="AA21">
-        <v>0.353658536585365</v>
+        <v>29</v>
       </c>
       <c r="AB21">
         <v>9.8706603131381802E-3</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="22" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B22">
         <v>82</v>
@@ -2874,22 +2874,22 @@
         <v>8218</v>
       </c>
       <c r="D22">
-        <v>110.865853658536</v>
+        <v>9091</v>
       </c>
       <c r="E22">
-        <v>29.8170731707317</v>
+        <v>2445</v>
       </c>
       <c r="F22">
-        <v>57.024390243902403</v>
+        <v>4676</v>
       </c>
       <c r="G22">
         <v>0.52288280581693702</v>
       </c>
       <c r="H22">
-        <v>11.8170731707317</v>
+        <v>969</v>
       </c>
       <c r="I22">
-        <v>33.975609756097498</v>
+        <v>2786</v>
       </c>
       <c r="J22">
         <v>0.34781048097631001</v>
@@ -2898,19 +2898,19 @@
         <v>0.35057887120115699</v>
       </c>
       <c r="L22">
-        <v>15.780487804878</v>
+        <v>1294</v>
       </c>
       <c r="M22">
-        <v>35.707317073170699</v>
+        <v>2928</v>
       </c>
       <c r="N22">
-        <v>23.9268292682926</v>
+        <v>1962</v>
       </c>
       <c r="O22">
-        <v>32.048780487804798</v>
+        <v>2628</v>
       </c>
       <c r="P22">
-        <v>3.4024390243902398</v>
+        <v>279</v>
       </c>
       <c r="Q22">
         <v>0.59877300613496898</v>
@@ -2934,16 +2934,16 @@
         <v>0.55170316301703104</v>
       </c>
       <c r="X22">
-        <v>5.5365853658536501</v>
+        <v>454</v>
       </c>
       <c r="Y22">
-        <v>5.59756097560975</v>
+        <v>459</v>
       </c>
       <c r="Z22">
         <v>9.8160821214713395E-2</v>
       </c>
       <c r="AA22">
-        <v>0.30487804878048702</v>
+        <v>25</v>
       </c>
       <c r="AB22">
         <v>8.9734386216798207E-3</v>
@@ -2951,7 +2951,7 @@
     </row>
     <row r="23" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B23">
         <v>82</v>
@@ -2960,22 +2960,22 @@
         <v>8233</v>
       </c>
       <c r="D23">
-        <v>111.890243902439</v>
+        <v>9175</v>
       </c>
       <c r="E23">
-        <v>26.3536585365853</v>
+        <v>2161</v>
       </c>
       <c r="F23">
-        <v>48.829268292682897</v>
+        <v>4004</v>
       </c>
       <c r="G23">
         <v>0.539710289710289</v>
       </c>
       <c r="H23">
-        <v>13.951219512195101</v>
+        <v>1144</v>
       </c>
       <c r="I23">
-        <v>39.841463414634099</v>
+        <v>3267</v>
       </c>
       <c r="J23">
         <v>0.35016835016835002</v>
@@ -2984,19 +2984,19 @@
         <v>0.35180055401662003</v>
       </c>
       <c r="L23">
-        <v>17.329268292682901</v>
+        <v>1421</v>
       </c>
       <c r="M23">
-        <v>28.048780487804802</v>
+        <v>2300</v>
       </c>
       <c r="N23">
-        <v>24.658536585365798</v>
+        <v>2022</v>
       </c>
       <c r="O23">
-        <v>34.5</v>
+        <v>2829</v>
       </c>
       <c r="P23">
-        <v>7.3536585365853604</v>
+        <v>603</v>
       </c>
       <c r="Q23">
         <v>0.53216103655714897</v>
@@ -3020,16 +3020,16 @@
         <v>0.56822418292531296</v>
       </c>
       <c r="X23">
-        <v>5.7804878048780397</v>
+        <v>474</v>
       </c>
       <c r="Y23">
-        <v>5.9146341463414602</v>
+        <v>485</v>
       </c>
       <c r="Z23">
         <v>0.121128871128871</v>
       </c>
       <c r="AA23">
-        <v>0.5</v>
+        <v>41</v>
       </c>
       <c r="AB23">
         <v>1.2549739822467E-2</v>
@@ -3037,7 +3037,7 @@
     </row>
     <row r="24" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B24">
         <v>82</v>
@@ -3046,22 +3046,22 @@
         <v>8030</v>
       </c>
       <c r="D24">
-        <v>112.87804878048701</v>
+        <v>9256</v>
       </c>
       <c r="E24">
-        <v>29.109756097560901</v>
+        <v>2387</v>
       </c>
       <c r="F24">
-        <v>52.890243902439003</v>
+        <v>4337</v>
       </c>
       <c r="G24">
         <v>0.55038044731381097</v>
       </c>
       <c r="H24">
-        <v>12.4634146341463</v>
+        <v>1022</v>
       </c>
       <c r="I24">
-        <v>33.390243902439003</v>
+        <v>2738</v>
       </c>
       <c r="J24">
         <v>0.37326515704893998</v>
@@ -3070,19 +3070,19 @@
         <v>0.37449615243679002</v>
       </c>
       <c r="L24">
-        <v>17.268292682926798</v>
+        <v>1416</v>
       </c>
       <c r="M24">
-        <v>31.951219512195099</v>
+        <v>2620</v>
       </c>
       <c r="N24">
-        <v>26.268292682926798</v>
+        <v>2154</v>
       </c>
       <c r="O24">
-        <v>27.585365853658502</v>
+        <v>2262</v>
       </c>
       <c r="P24">
-        <v>9.8048780487804805</v>
+        <v>804</v>
       </c>
       <c r="Q24">
         <v>0.54880603267700001</v>
@@ -3106,16 +3106,16 @@
         <v>0.58946830265848604</v>
       </c>
       <c r="X24">
-        <v>5.3170731707316996</v>
+        <v>436</v>
       </c>
       <c r="Y24">
-        <v>4.0121951219512102</v>
+        <v>329</v>
       </c>
       <c r="Z24">
         <v>7.5858888632695395E-2</v>
       </c>
       <c r="AA24">
-        <v>0.28048780487804797</v>
+        <v>23</v>
       </c>
       <c r="AB24">
         <v>8.4002921840759595E-3</v>
@@ -3123,7 +3123,7 @@
     </row>
     <row r="25" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B25">
         <v>82</v>
@@ -3132,22 +3132,22 @@
         <v>7995</v>
       </c>
       <c r="D25">
-        <v>113.390243902439</v>
+        <v>9298</v>
       </c>
       <c r="E25">
-        <v>27.609756097560901</v>
+        <v>2264</v>
       </c>
       <c r="F25">
-        <v>49.097560975609703</v>
+        <v>4026</v>
       </c>
       <c r="G25">
         <v>0.56234475906606995</v>
       </c>
       <c r="H25">
-        <v>13.3170731707317</v>
+        <v>1092</v>
       </c>
       <c r="I25">
-        <v>36.3536585365853</v>
+        <v>2981</v>
       </c>
       <c r="J25">
         <v>0.36632002683663201</v>
@@ -3156,19 +3156,19 @@
         <v>0.369043595809395</v>
       </c>
       <c r="L25">
-        <v>18.219512195121901</v>
+        <v>1494</v>
       </c>
       <c r="M25">
-        <v>30.634146341463399</v>
+        <v>2512</v>
       </c>
       <c r="N25">
-        <v>24.585365853658502</v>
+        <v>2016</v>
       </c>
       <c r="O25">
-        <v>32.012195121951201</v>
+        <v>2625</v>
       </c>
       <c r="P25">
-        <v>7.9390243902439002</v>
+        <v>651</v>
       </c>
       <c r="Q25">
         <v>0.55477031802120103</v>
@@ -3192,16 +3192,16 @@
         <v>0.59219269102990002</v>
       </c>
       <c r="X25">
-        <v>3.9024390243902398</v>
+        <v>320</v>
       </c>
       <c r="Y25">
-        <v>3.8902439024390199</v>
+        <v>319</v>
       </c>
       <c r="Z25">
         <v>7.9234972677595605E-2</v>
       </c>
       <c r="AA25">
-        <v>0.30487804878048702</v>
+        <v>25</v>
       </c>
       <c r="AB25">
         <v>8.3864475008386397E-3</v>
@@ -3209,7 +3209,7 @@
     </row>
     <row r="26" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B26">
         <v>82</v>
@@ -3218,22 +3218,22 @@
         <v>8021</v>
       </c>
       <c r="D26">
-        <v>114.292682926829</v>
+        <v>9372</v>
       </c>
       <c r="E26">
-        <v>25.987804878048699</v>
+        <v>2131</v>
       </c>
       <c r="F26">
-        <v>47.731707317073102</v>
+        <v>3914</v>
       </c>
       <c r="G26">
         <v>0.54445579969340796</v>
       </c>
       <c r="H26">
-        <v>15.0365853658536</v>
+        <v>1233</v>
       </c>
       <c r="I26">
-        <v>39.865853658536501</v>
+        <v>3269</v>
       </c>
       <c r="J26">
         <v>0.37717956561639598</v>
@@ -3242,19 +3242,19 @@
         <v>0.38008631319358799</v>
       </c>
       <c r="L26">
-        <v>17.207317073170699</v>
+        <v>1411</v>
       </c>
       <c r="M26">
-        <v>28.731707317073099</v>
+        <v>2356</v>
       </c>
       <c r="N26">
-        <v>23.2439024390243</v>
+        <v>1906</v>
       </c>
       <c r="O26">
-        <v>35.268292682926798</v>
+        <v>2892</v>
       </c>
       <c r="P26">
-        <v>9.8414634146341395</v>
+        <v>807</v>
       </c>
       <c r="Q26">
         <v>0.55279211637728698</v>
@@ -3278,16 +3278,16 @@
         <v>0.58688545203067999</v>
       </c>
       <c r="X26">
-        <v>5.2926829268292597</v>
+        <v>434</v>
       </c>
       <c r="Y26">
-        <v>4.2439024390243896</v>
+        <v>348</v>
       </c>
       <c r="Z26">
         <v>8.8911599386816503E-2</v>
       </c>
       <c r="AA26">
-        <v>0.24390243902438999</v>
+        <v>20</v>
       </c>
       <c r="AB26">
         <v>6.1180789232180999E-3</v>
@@ -3295,7 +3295,7 @@
     </row>
     <row r="27" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B27">
         <v>82</v>
@@ -3304,22 +3304,22 @@
         <v>7883</v>
       </c>
       <c r="D27">
-        <v>105.10975609755999</v>
+        <v>8619</v>
       </c>
       <c r="E27">
-        <v>24.060975609756099</v>
+        <v>1973</v>
       </c>
       <c r="F27">
-        <v>46.682926829268197</v>
+        <v>3828</v>
       </c>
       <c r="G27">
         <v>0.51541274817136795</v>
       </c>
       <c r="H27">
-        <v>13.5731707317073</v>
+        <v>1113</v>
       </c>
       <c r="I27">
-        <v>39.414634146341399</v>
+        <v>3232</v>
       </c>
       <c r="J27">
         <v>0.34436881188118801</v>
@@ -3328,19 +3328,19 @@
         <v>0.34597451041342803</v>
       </c>
       <c r="L27">
-        <v>16.268292682926798</v>
+        <v>1334</v>
       </c>
       <c r="M27">
-        <v>25.975609756097501</v>
+        <v>2130</v>
       </c>
       <c r="N27">
-        <v>22.146341463414601</v>
+        <v>1816</v>
       </c>
       <c r="O27">
-        <v>36.512195121951201</v>
+        <v>2994</v>
       </c>
       <c r="P27">
-        <v>4.2073170731707297</v>
+        <v>345</v>
       </c>
       <c r="Q27">
         <v>0.53978712620375002</v>
@@ -3364,16 +3364,16 @@
         <v>0.55048755452912501</v>
       </c>
       <c r="X27">
-        <v>4.7560975609755998</v>
+        <v>390</v>
       </c>
       <c r="Y27">
-        <v>5.1097560975609699</v>
+        <v>419</v>
       </c>
       <c r="Z27">
         <v>0.109456635318704</v>
       </c>
       <c r="AA27">
-        <v>0.46341463414634099</v>
+        <v>38</v>
       </c>
       <c r="AB27">
         <v>1.17574257425742E-2</v>
@@ -3381,7 +3381,7 @@
     </row>
     <row r="28" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B28">
         <v>82</v>
@@ -3390,22 +3390,22 @@
         <v>7846</v>
       </c>
       <c r="D28">
-        <v>105.37804878048701</v>
+        <v>8641</v>
       </c>
       <c r="E28">
-        <v>26.914634146341399</v>
+        <v>2207</v>
       </c>
       <c r="F28">
-        <v>50.5</v>
+        <v>4141</v>
       </c>
       <c r="G28">
         <v>0.53296305240280095</v>
       </c>
       <c r="H28">
-        <v>11.2317073170731</v>
+        <v>921</v>
       </c>
       <c r="I28">
-        <v>35.268292682926798</v>
+        <v>2892</v>
       </c>
       <c r="J28">
         <v>0.31846473029045602</v>
@@ -3414,19 +3414,19 @@
         <v>0.32112970711297001</v>
       </c>
       <c r="L28">
-        <v>17.8536585365853</v>
+        <v>1464</v>
       </c>
       <c r="M28">
-        <v>27.219512195121901</v>
+        <v>2232</v>
       </c>
       <c r="N28">
-        <v>26.609756097560901</v>
+        <v>2182</v>
       </c>
       <c r="O28">
-        <v>28.207317073170699</v>
+        <v>2313</v>
       </c>
       <c r="P28">
-        <v>5.48780487804878</v>
+        <v>450</v>
       </c>
       <c r="Q28">
         <v>0.50566379700951503</v>
@@ -3450,16 +3450,16 @@
         <v>0.54810142711518794</v>
       </c>
       <c r="X28">
-        <v>4.7317073170731696</v>
+        <v>388</v>
       </c>
       <c r="Y28">
-        <v>4.2195121951219496</v>
+        <v>346</v>
       </c>
       <c r="Z28">
         <v>8.3554696933107894E-2</v>
       </c>
       <c r="AA28">
-        <v>0.18292682926829201</v>
+        <v>15</v>
       </c>
       <c r="AB28">
         <v>5.1867219917012403E-3</v>
@@ -3467,7 +3467,7 @@
     </row>
     <row r="29" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B29">
         <v>82</v>
@@ -3476,22 +3476,22 @@
         <v>8042</v>
       </c>
       <c r="D29">
-        <v>113.621951219512</v>
+        <v>9317</v>
       </c>
       <c r="E29">
-        <v>26.890243902439</v>
+        <v>2205</v>
       </c>
       <c r="F29">
-        <v>48.329268292682897</v>
+        <v>3963</v>
       </c>
       <c r="G29">
         <v>0.55639666919000696</v>
       </c>
       <c r="H29">
-        <v>14.3414634146341</v>
+        <v>1176</v>
       </c>
       <c r="I29">
-        <v>37.951219512195102</v>
+        <v>3112</v>
       </c>
       <c r="J29">
         <v>0.37789203084832901</v>
@@ -3500,19 +3500,19 @@
         <v>0.37886597938144301</v>
       </c>
       <c r="L29">
-        <v>16.8170731707317</v>
+        <v>1379</v>
       </c>
       <c r="M29">
-        <v>30.024390243902399</v>
+        <v>2462</v>
       </c>
       <c r="N29">
-        <v>23.756097560975601</v>
+        <v>1948</v>
       </c>
       <c r="O29">
-        <v>38.268292682926798</v>
+        <v>3138</v>
       </c>
       <c r="P29">
-        <v>4.7560975609755998</v>
+        <v>390</v>
       </c>
       <c r="Q29">
         <v>0.55827664399092902</v>
@@ -3536,16 +3536,16 @@
         <v>0.59395372619199704</v>
       </c>
       <c r="X29">
-        <v>3.5121951219512102</v>
+        <v>288</v>
       </c>
       <c r="Y29">
-        <v>3.6341463414634099</v>
+        <v>298</v>
       </c>
       <c r="Z29">
         <v>7.5195558920009994E-2</v>
       </c>
       <c r="AA29">
-        <v>0.37804878048780399</v>
+        <v>31</v>
       </c>
       <c r="AB29">
         <v>9.9614395886889404E-3</v>
@@ -3553,7 +3553,7 @@
     </row>
     <row r="30" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B30">
         <v>82</v>
@@ -3562,22 +3562,22 @@
         <v>8131</v>
       </c>
       <c r="D30">
-        <v>110.84146341463401</v>
+        <v>9089</v>
       </c>
       <c r="E30">
-        <v>27.634146341463399</v>
+        <v>2266</v>
       </c>
       <c r="F30">
-        <v>52.414634146341399</v>
+        <v>4298</v>
       </c>
       <c r="G30">
         <v>0.52722196370404795</v>
       </c>
       <c r="H30">
-        <v>12.890243902439</v>
+        <v>1057</v>
       </c>
       <c r="I30">
-        <v>37.743902439024303</v>
+        <v>3095</v>
       </c>
       <c r="J30">
         <v>0.34151857835218002</v>
@@ -3586,19 +3586,19 @@
         <v>0.34307992202728999</v>
       </c>
       <c r="L30">
-        <v>16.902439024390201</v>
+        <v>1386</v>
       </c>
       <c r="M30">
-        <v>26.560975609756099</v>
+        <v>2178</v>
       </c>
       <c r="N30">
-        <v>28.707317073170699</v>
+        <v>2354</v>
       </c>
       <c r="O30">
-        <v>31.5731707317073</v>
+        <v>2589</v>
       </c>
       <c r="P30">
-        <v>7.09756097560975</v>
+        <v>582</v>
       </c>
       <c r="Q30">
         <v>0.480582524271844</v>
@@ -3622,16 +3622,16 @@
         <v>0.55422423279129396</v>
       </c>
       <c r="X30">
-        <v>6.7560975609755998</v>
+        <v>554</v>
       </c>
       <c r="Y30">
-        <v>5.2195121951219496</v>
+        <v>428</v>
       </c>
       <c r="Z30">
         <v>9.9581200558399197E-2</v>
       </c>
       <c r="AA30">
-        <v>0.30487804878048702</v>
+        <v>25</v>
       </c>
       <c r="AB30">
         <v>8.0775444264943406E-3</v>
@@ -3639,7 +3639,7 @@
     </row>
     <row r="31" spans="1:28" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B31">
         <v>82</v>
@@ -3648,22 +3648,22 @@
         <v>8162</v>
       </c>
       <c r="D31">
-        <v>113.87804878048701</v>
+        <v>9338</v>
       </c>
       <c r="E31">
-        <v>27.634146341463399</v>
+        <v>2266</v>
       </c>
       <c r="F31">
-        <v>50.146341463414601</v>
+        <v>4112</v>
       </c>
       <c r="G31">
         <v>0.55107003891050499</v>
       </c>
       <c r="H31">
-        <v>14.1219512195121</v>
+        <v>1158</v>
       </c>
       <c r="I31">
-        <v>39.597560975609703</v>
+        <v>3247</v>
       </c>
       <c r="J31">
         <v>0.35663689559593398</v>
@@ -3672,19 +3672,19 @@
         <v>0.35844961240310003</v>
       </c>
       <c r="L31">
-        <v>16.2439024390243</v>
+        <v>1332</v>
       </c>
       <c r="M31">
-        <v>32.9268292682926</v>
+        <v>2700</v>
       </c>
       <c r="N31">
-        <v>22.341463414634099</v>
+        <v>1832</v>
       </c>
       <c r="O31">
-        <v>36.512195121951201</v>
+        <v>2994</v>
       </c>
       <c r="P31">
-        <v>5.8536585365853604</v>
+        <v>480</v>
       </c>
       <c r="Q31">
         <v>0.595763459841129</v>
@@ -3708,16 +3708,16 @@
         <v>0.57544488383588699</v>
       </c>
       <c r="X31">
-        <v>4.5609756097560901</v>
+        <v>374</v>
       </c>
       <c r="Y31">
-        <v>4.0487804878048701</v>
+        <v>332</v>
       </c>
       <c r="Z31">
         <v>8.0739299610894905E-2</v>
       </c>
       <c r="AA31">
-        <v>0.292682926829268</v>
+        <v>24</v>
       </c>
       <c r="AB31">
         <v>7.3914382506929397E-3</v>

</xml_diff>